<commit_message>
feat: Thêm cột CTR cho Group A, cột Source cho Group B với logic mapping mới, và cập nhật cấu trúc file Excel đầu ra.
</commit_message>
<xml_diff>
--- a/destination/Tam Đảo - keyword.xlsx
+++ b/destination/Tam Đảo - keyword.xlsx
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I136"/>
+  <dimension ref="A1:J139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -509,8 +509,9 @@
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -530,14 +531,14 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>- Mục tiêu: Chiếm lĩnh thị trường du lịch Tam Đảo cho vietgoing.com bằng dữ liệu thực tế (GSC) + xu hướng (SEO Insider) + thị trường (Google Planner).</t>
+          <t>- Mục tiêu: Chiếm lĩnh thị trường du lịch Tam Đảo cho vietgoing.com bằng dữ liệu thực tế (GSC) + xu hướng (Trend/SEO Insider).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>- Tổng số từ khóa: 100</t>
+          <t>- Tổng số từ khóa: 101</t>
         </is>
       </c>
     </row>
@@ -551,21 +552,21 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>- data/google_search_console/Queries.csv (48 từ khóa — Group A)</t>
+          <t>- data/google_search_console/Queries.csv (48 từ khóa)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>- data/seo_insider/advance_search_report.csv (11 từ khóa — Group B)</t>
+          <t>- web (tam-dao.csv) (42 từ khóa)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>- data/google_planner/tamdao/ (41 từ khóa — Group B, lọc từ 531 keywords thô)</t>
+          <t>- data/seo_insider/advance_search_report.csv (11 từ khóa)</t>
         </is>
       </c>
     </row>
@@ -614,6 +615,11 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
+          <t>CTR</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
           <t>source</t>
         </is>
       </c>
@@ -656,6 +662,11 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
+          <t>16.94%</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -698,6 +709,11 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
+          <t>11.11%</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -740,6 +756,11 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
+          <t>9.6%</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -782,6 +803,11 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
+          <t>8.33%</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -824,6 +850,11 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
+          <t>7.05%</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -866,6 +897,11 @@
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
+          <t>6.96%</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -908,6 +944,11 @@
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
+          <t>6.75%</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -950,6 +991,11 @@
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
+          <t>6.75%</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -992,6 +1038,11 @@
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
+          <t>6.54%</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -1034,6 +1085,11 @@
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
+          <t>6.15%</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -1076,6 +1132,11 @@
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
+          <t>5.99%</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -1118,6 +1179,11 @@
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
+          <t>5.77%</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -1160,6 +1226,11 @@
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
+          <t>5.68%</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -1202,6 +1273,11 @@
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
+          <t>4.58%</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -1244,6 +1320,11 @@
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
+          <t>4.12%</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -1286,6 +1367,11 @@
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
+          <t>3.92%</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -1328,6 +1414,11 @@
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
+          <t>3.62%</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -1370,6 +1461,11 @@
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
+          <t>3.58%</t>
+        </is>
+      </c>
+      <c r="I30" s="6" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -1412,6 +1508,11 @@
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
+          <t>3.48%</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -1454,6 +1555,11 @@
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
+          <t>3.29%</t>
+        </is>
+      </c>
+      <c r="I32" s="6" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -1496,6 +1602,11 @@
       </c>
       <c r="H33" s="5" t="inlineStr">
         <is>
+          <t>3.28%</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -1538,6 +1649,11 @@
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
+          <t>3.25%</t>
+        </is>
+      </c>
+      <c r="I34" s="6" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -1580,6 +1696,11 @@
       </c>
       <c r="H35" s="5" t="inlineStr">
         <is>
+          <t>3.06%</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -1622,6 +1743,11 @@
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
+          <t>2.89%</t>
+        </is>
+      </c>
+      <c r="I36" s="6" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -1664,6 +1790,11 @@
       </c>
       <c r="H37" s="5" t="inlineStr">
         <is>
+          <t>2.81%</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -1706,6 +1837,11 @@
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
+          <t>2.78%</t>
+        </is>
+      </c>
+      <c r="I38" s="6" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -1748,6 +1884,11 @@
       </c>
       <c r="H39" s="5" t="inlineStr">
         <is>
+          <t>2.76%</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -1790,6 +1931,11 @@
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
+          <t>2.75%</t>
+        </is>
+      </c>
+      <c r="I40" s="6" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -1832,6 +1978,11 @@
       </c>
       <c r="H41" s="5" t="inlineStr">
         <is>
+          <t>2.55%</t>
+        </is>
+      </c>
+      <c r="I41" s="5" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -1874,6 +2025,11 @@
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
+          <t>2.23%</t>
+        </is>
+      </c>
+      <c r="I42" s="6" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -1916,6 +2072,11 @@
       </c>
       <c r="H43" s="5" t="inlineStr">
         <is>
+          <t>2.08%</t>
+        </is>
+      </c>
+      <c r="I43" s="5" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -1958,6 +2119,11 @@
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
+          <t>2.07%</t>
+        </is>
+      </c>
+      <c r="I44" s="6" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -2000,6 +2166,11 @@
       </c>
       <c r="H45" s="5" t="inlineStr">
         <is>
+          <t>2.02%</t>
+        </is>
+      </c>
+      <c r="I45" s="5" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -2042,6 +2213,11 @@
       </c>
       <c r="H46" s="6" t="inlineStr">
         <is>
+          <t>2.0%</t>
+        </is>
+      </c>
+      <c r="I46" s="6" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -2084,6 +2260,11 @@
       </c>
       <c r="H47" s="5" t="inlineStr">
         <is>
+          <t>1.96%</t>
+        </is>
+      </c>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -2126,6 +2307,11 @@
       </c>
       <c r="H48" s="6" t="inlineStr">
         <is>
+          <t>1.84%</t>
+        </is>
+      </c>
+      <c r="I48" s="6" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -2153,7 +2339,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>Commercial Investigation</t>
+          <t>Transaction</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
@@ -2167,6 +2353,11 @@
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t>1.83%</t>
+        </is>
+      </c>
+      <c r="I49" s="5" t="inlineStr">
         <is>
           <t>GSC Vietgoing.com</t>
         </is>
@@ -2210,6 +2401,11 @@
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
+          <t>1.63%</t>
+        </is>
+      </c>
+      <c r="I50" s="6" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -2237,7 +2433,7 @@
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>Commercial Investigation</t>
+          <t>Transaction</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
@@ -2251,6 +2447,11 @@
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">
+        <is>
+          <t>1.57%</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="inlineStr">
         <is>
           <t>GSC Vietgoing.com</t>
         </is>
@@ -2294,6 +2495,11 @@
       </c>
       <c r="H52" s="6" t="inlineStr">
         <is>
+          <t>1.47%</t>
+        </is>
+      </c>
+      <c r="I52" s="6" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -2336,6 +2542,11 @@
       </c>
       <c r="H53" s="5" t="inlineStr">
         <is>
+          <t>1.37%</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -2378,6 +2589,11 @@
       </c>
       <c r="H54" s="6" t="inlineStr">
         <is>
+          <t>1.3%</t>
+        </is>
+      </c>
+      <c r="I54" s="6" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -2420,6 +2636,11 @@
       </c>
       <c r="H55" s="5" t="inlineStr">
         <is>
+          <t>1.21%</t>
+        </is>
+      </c>
+      <c r="I55" s="5" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -2462,6 +2683,11 @@
       </c>
       <c r="H56" s="6" t="inlineStr">
         <is>
+          <t>1.18%</t>
+        </is>
+      </c>
+      <c r="I56" s="6" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -2504,6 +2730,11 @@
       </c>
       <c r="H57" s="5" t="inlineStr">
         <is>
+          <t>1.12%</t>
+        </is>
+      </c>
+      <c r="I57" s="5" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -2546,6 +2777,11 @@
       </c>
       <c r="H58" s="6" t="inlineStr">
         <is>
+          <t>1.08%</t>
+        </is>
+      </c>
+      <c r="I58" s="6" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -2588,6 +2824,11 @@
       </c>
       <c r="H59" s="5" t="inlineStr">
         <is>
+          <t>0.83%</t>
+        </is>
+      </c>
+      <c r="I59" s="5" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -2630,6 +2871,11 @@
       </c>
       <c r="H60" s="6" t="inlineStr">
         <is>
+          <t>0.74%</t>
+        </is>
+      </c>
+      <c r="I60" s="6" t="inlineStr">
+        <is>
           <t>GSC Vietgoing.com</t>
         </is>
       </c>
@@ -2687,6 +2933,11 @@
           <t>bid (high)</t>
         </is>
       </c>
+      <c r="J63" s="7" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
@@ -2734,6 +2985,11 @@
           <t>0 VNĐ</t>
         </is>
       </c>
+      <c r="J64" s="5" t="inlineStr">
+        <is>
+          <t>Seo Insider</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
@@ -2781,6 +3037,11 @@
           <t>0 VNĐ</t>
         </is>
       </c>
+      <c r="J65" s="6" t="inlineStr">
+        <is>
+          <t>Seo Insider</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
@@ -2828,6 +3089,11 @@
           <t>0 VNĐ</t>
         </is>
       </c>
+      <c r="J66" s="5" t="inlineStr">
+        <is>
+          <t>Seo Insider</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
@@ -2875,6 +3141,11 @@
           <t>0 VNĐ</t>
         </is>
       </c>
+      <c r="J67" s="6" t="inlineStr">
+        <is>
+          <t>Seo Insider</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
@@ -2922,6 +3193,11 @@
           <t>0 VNĐ</t>
         </is>
       </c>
+      <c r="J68" s="5" t="inlineStr">
+        <is>
+          <t>Seo Insider</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
@@ -2969,6 +3245,11 @@
           <t>0 VNĐ</t>
         </is>
       </c>
+      <c r="J69" s="6" t="inlineStr">
+        <is>
+          <t>Seo Insider</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
@@ -3016,6 +3297,11 @@
           <t>0 VNĐ</t>
         </is>
       </c>
+      <c r="J70" s="5" t="inlineStr">
+        <is>
+          <t>Seo Insider</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
@@ -3063,6 +3349,11 @@
           <t>0 VNĐ</t>
         </is>
       </c>
+      <c r="J71" s="6" t="inlineStr">
+        <is>
+          <t>Seo Insider</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
@@ -3110,6 +3401,11 @@
           <t>0 VNĐ</t>
         </is>
       </c>
+      <c r="J72" s="5" t="inlineStr">
+        <is>
+          <t>Seo Insider</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
@@ -3157,6 +3453,11 @@
           <t>0 VNĐ</t>
         </is>
       </c>
+      <c r="J73" s="6" t="inlineStr">
+        <is>
+          <t>Seo Insider</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
@@ -3204,6 +3505,11 @@
           <t>0 VNĐ</t>
         </is>
       </c>
+      <c r="J74" s="5" t="inlineStr">
+        <is>
+          <t>Seo Insider</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
@@ -3213,7 +3519,7 @@
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>Khách sạn Tam Đảo</t>
+          <t>Homestay Tam Đảo</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
@@ -3223,17 +3529,17 @@
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>khách sạn tam đảo</t>
+          <t>homestay tam đảo giá rẻ</t>
         </is>
       </c>
       <c r="E75" s="6" t="inlineStr">
         <is>
-          <t>Commercial Investigation</t>
+          <t>Transaction</t>
         </is>
       </c>
       <c r="F75" s="6" t="inlineStr">
         <is>
-          <t>5000</t>
+          <t>400</t>
         </is>
       </c>
       <c r="G75" s="6" t="inlineStr">
@@ -3243,12 +3549,17 @@
       </c>
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I75" s="6" t="inlineStr">
         <is>
-          <t>2.435 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J75" s="6" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -3260,7 +3571,7 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>Khách sạn Tam Đảo</t>
+          <t>Homestay Tam Đảo</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
@@ -3270,17 +3581,17 @@
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>venus hotel tam đảo</t>
+          <t>booking homestay tam đảo</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t>Commercial Investigation</t>
+          <t>Transaction</t>
         </is>
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>5000</t>
+          <t>200</t>
         </is>
       </c>
       <c r="G76" s="5" t="inlineStr">
@@ -3290,12 +3601,17 @@
       </c>
       <c r="H76" s="5" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I76" s="5" t="inlineStr">
         <is>
-          <t>2.642 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J76" s="5" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -3307,7 +3623,7 @@
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>Khách sạn Tam Đảo</t>
+          <t>Homestay Tam Đảo</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
@@ -3317,7 +3633,7 @@
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>hotel tam đảo</t>
+          <t>homestay tam đảo có hồ bơi</t>
         </is>
       </c>
       <c r="E77" s="6" t="inlineStr">
@@ -3327,7 +3643,7 @@
       </c>
       <c r="F77" s="6" t="inlineStr">
         <is>
-          <t>5000</t>
+          <t>300</t>
         </is>
       </c>
       <c r="G77" s="6" t="inlineStr">
@@ -3337,12 +3653,17 @@
       </c>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I77" s="6" t="inlineStr">
         <is>
-          <t>2.799 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J77" s="6" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -3354,27 +3675,27 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>Địa danh Tam Đảo</t>
+          <t>Hà Nội Trip</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>Địa danh tham quan</t>
+          <t>Lưu trú</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>cổng trời tam đảo</t>
+          <t>khách sạn hà nội đi tam đảo</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Commercial Investigation</t>
         </is>
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>5000</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G78" s="5" t="inlineStr">
@@ -3384,12 +3705,17 @@
       </c>
       <c r="H78" s="5" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I78" s="5" t="inlineStr">
         <is>
           <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J78" s="5" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -3401,7 +3727,7 @@
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>Đặt phòng Tam Đảo</t>
+          <t>Hà Nội Trip</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
@@ -3411,17 +3737,17 @@
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>đặt phòng tam đảo</t>
+          <t>homestay hà nội đi tam đảo</t>
         </is>
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>Transaction</t>
+          <t>Commercial Investigation</t>
         </is>
       </c>
       <c r="F79" s="6" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G79" s="6" t="inlineStr">
@@ -3431,12 +3757,17 @@
       </c>
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I79" s="6" t="inlineStr">
         <is>
-          <t>3.666 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J79" s="6" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -3448,7 +3779,7 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>Đặt phòng Tam Đảo</t>
+          <t>Khách sạn 5 sao Tam Đảo</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
@@ -3458,17 +3789,17 @@
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>book phòng tam đảo</t>
+          <t>khách sạn 5 sao tam đảo</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t>Transaction</t>
+          <t>Commercial Investigation</t>
         </is>
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>400</t>
         </is>
       </c>
       <c r="G80" s="5" t="inlineStr">
@@ -3478,12 +3809,17 @@
       </c>
       <c r="H80" s="5" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I80" s="5" t="inlineStr">
         <is>
-          <t>3.116 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J80" s="5" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -3495,7 +3831,7 @@
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>Đặt phòng Tam Đảo</t>
+          <t>Khách sạn Tam Đảo</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
@@ -3505,7 +3841,7 @@
       </c>
       <c r="D81" s="6" t="inlineStr">
         <is>
-          <t>booking tam đảo</t>
+          <t>khách sạn venus tam đảo giá rẻ</t>
         </is>
       </c>
       <c r="E81" s="6" t="inlineStr">
@@ -3515,7 +3851,7 @@
       </c>
       <c r="F81" s="6" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G81" s="6" t="inlineStr">
@@ -3525,12 +3861,17 @@
       </c>
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I81" s="6" t="inlineStr">
         <is>
-          <t>2.689 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J81" s="6" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -3552,7 +3893,7 @@
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>khách sạn trung tâm tam đảo</t>
+          <t>khách sạn đẹp tam đảo</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -3562,7 +3903,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>300</t>
         </is>
       </c>
       <c r="G82" s="5" t="inlineStr">
@@ -3572,12 +3913,17 @@
       </c>
       <c r="H82" s="5" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I82" s="5" t="inlineStr">
         <is>
-          <t>2.962 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J82" s="5" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -3599,7 +3945,7 @@
       </c>
       <c r="D83" s="6" t="inlineStr">
         <is>
-          <t>khách sạn đẹp nhất tam đảo</t>
+          <t>đặt phòng khách sạn tam đảo</t>
         </is>
       </c>
       <c r="E83" s="6" t="inlineStr">
@@ -3619,12 +3965,17 @@
       </c>
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I83" s="6" t="inlineStr">
         <is>
-          <t>1.885 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J83" s="6" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -3646,7 +3997,7 @@
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>khách sạn tam đảo 5 sao</t>
+          <t>hotel tam đảo sạch sẽ</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -3656,7 +4007,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>200</t>
         </is>
       </c>
       <c r="G84" s="5" t="inlineStr">
@@ -3666,12 +4017,17 @@
       </c>
       <c r="H84" s="5" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I84" s="5" t="inlineStr">
         <is>
-          <t>2.312 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J84" s="5" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -3683,7 +4039,7 @@
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>Khách sạn Tam Đảo</t>
+          <t>Resort Tam Đảo</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
@@ -3693,7 +4049,7 @@
       </c>
       <c r="D85" s="6" t="inlineStr">
         <is>
-          <t>khách sạn đẹp ở tam đảo</t>
+          <t>resort tam đảo nghỉ dưỡng</t>
         </is>
       </c>
       <c r="E85" s="6" t="inlineStr">
@@ -3703,7 +4059,7 @@
       </c>
       <c r="F85" s="6" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>200</t>
         </is>
       </c>
       <c r="G85" s="6" t="inlineStr">
@@ -3713,12 +4069,17 @@
       </c>
       <c r="H85" s="6" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I85" s="6" t="inlineStr">
         <is>
-          <t>1.818 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J85" s="6" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -3730,7 +4091,7 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>Khách sạn Tam Đảo</t>
+          <t>Resort Tam Đảo</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
@@ -3740,7 +4101,7 @@
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>khách sạn tại tam đảo</t>
+          <t>review resort tam đảo</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -3750,7 +4111,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>200</t>
         </is>
       </c>
       <c r="G86" s="5" t="inlineStr">
@@ -3760,12 +4121,17 @@
       </c>
       <c r="H86" s="5" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I86" s="5" t="inlineStr">
         <is>
-          <t>2.101 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J86" s="5" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -3777,27 +4143,27 @@
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>Khách sạn Tam Đảo</t>
+          <t>Di chuyển Tam Đảo</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>Lưu trú</t>
+          <t>Di chuyển</t>
         </is>
       </c>
       <c r="D87" s="6" t="inlineStr">
         <is>
-          <t>khách sạn ở tam đảo gần trung tâm</t>
+          <t>xe taxi đi tam đảo</t>
         </is>
       </c>
       <c r="E87" s="6" t="inlineStr">
         <is>
-          <t>Commercial Investigation</t>
+          <t>Transaction</t>
         </is>
       </c>
       <c r="F87" s="6" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G87" s="6" t="inlineStr">
@@ -3807,12 +4173,17 @@
       </c>
       <c r="H87" s="6" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I87" s="6" t="inlineStr">
         <is>
-          <t>1.706 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J87" s="6" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -3824,27 +4195,27 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>Khách sạn Tam Đảo</t>
+          <t>Di chuyển Tam Đảo</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>Lưu trú</t>
+          <t>Di chuyển</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>khách sạn ở tam đảo</t>
+          <t>thuê xe máy tam đảo</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t>Commercial Investigation</t>
+          <t>Transaction</t>
         </is>
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>300</t>
         </is>
       </c>
       <c r="G88" s="5" t="inlineStr">
@@ -3854,12 +4225,17 @@
       </c>
       <c r="H88" s="5" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I88" s="5" t="inlineStr">
         <is>
-          <t>2.167 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J88" s="5" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -3871,17 +4247,17 @@
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>Đặt phòng Tam Đảo</t>
+          <t>Di chuyển Tam Đảo</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>Lưu trú</t>
+          <t>Di chuyển</t>
         </is>
       </c>
       <c r="D89" s="6" t="inlineStr">
         <is>
-          <t>phòng tam đảo</t>
+          <t>đặt vé xe đi tam đảo</t>
         </is>
       </c>
       <c r="E89" s="6" t="inlineStr">
@@ -3891,7 +4267,7 @@
       </c>
       <c r="F89" s="6" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G89" s="6" t="inlineStr">
@@ -3901,12 +4277,17 @@
       </c>
       <c r="H89" s="6" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I89" s="6" t="inlineStr">
         <is>
-          <t>2.436 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J89" s="6" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -3918,27 +4299,27 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>Khách sạn Tam Đảo</t>
+          <t>Di chuyển Tam Đảo</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>Lưu trú</t>
+          <t>Di chuyển</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>ks tam đảo</t>
+          <t>vé xe giường nằm đi tam đảo</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t>Commercial Investigation</t>
+          <t>Transaction</t>
         </is>
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>100</t>
         </is>
       </c>
       <c r="G90" s="5" t="inlineStr">
@@ -3948,12 +4329,17 @@
       </c>
       <c r="H90" s="5" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I90" s="5" t="inlineStr">
         <is>
-          <t>3.266 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J90" s="5" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -3965,27 +4351,27 @@
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>Khách sạn Tam Đảo</t>
+          <t>Di chuyển Tam Đảo</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>Lưu trú</t>
+          <t>Di chuyển</t>
         </is>
       </c>
       <c r="D91" s="6" t="inlineStr">
         <is>
-          <t>khách sạn nam á tam đảo</t>
+          <t>đặt vé xe limosine tam đảo</t>
         </is>
       </c>
       <c r="E91" s="6" t="inlineStr">
         <is>
-          <t>Commercial Investigation</t>
+          <t>Transaction</t>
         </is>
       </c>
       <c r="F91" s="6" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G91" s="6" t="inlineStr">
@@ -3995,12 +4381,17 @@
       </c>
       <c r="H91" s="6" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I91" s="6" t="inlineStr">
         <is>
-          <t>1.529 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J91" s="6" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -4012,17 +4403,17 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>Khách sạn Tam Đảo</t>
+          <t>Di chuyển Tam Đảo</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>Lưu trú</t>
+          <t>Di chuyển</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>khách sạn anh minh tam đảo</t>
+          <t>kinh nghiệm đi phượt xe máy tam đảo</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -4032,7 +4423,7 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>200</t>
         </is>
       </c>
       <c r="G92" s="5" t="inlineStr">
@@ -4042,12 +4433,17 @@
       </c>
       <c r="H92" s="5" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I92" s="5" t="inlineStr">
         <is>
-          <t>2.078 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J92" s="5" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -4059,17 +4455,17 @@
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>Khách sạn Tam Đảo</t>
+          <t>Di chuyển Tam Đảo</t>
         </is>
       </c>
       <c r="C93" s="6" t="inlineStr">
         <is>
-          <t>Lưu trú</t>
+          <t>Di chuyển</t>
         </is>
       </c>
       <c r="D93" s="6" t="inlineStr">
         <is>
-          <t>khách sạn century tam đảo</t>
+          <t>địa điểm phượt tam đảo bằng xe máy</t>
         </is>
       </c>
       <c r="E93" s="6" t="inlineStr">
@@ -4079,7 +4475,7 @@
       </c>
       <c r="F93" s="6" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>200</t>
         </is>
       </c>
       <c r="G93" s="6" t="inlineStr">
@@ -4089,12 +4485,17 @@
       </c>
       <c r="H93" s="6" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I93" s="6" t="inlineStr">
         <is>
-          <t>1.102 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J93" s="6" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -4106,27 +4507,27 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>Khách sạn Tam Đảo</t>
+          <t>Hà Nội Trip</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>Lưu trú</t>
+          <t>Di chuyển</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>khách sạn 5 sao tam đảo</t>
+          <t>tour du lịch hà nội tam đảo 2 ngày 1 đêm</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t>Commercial Investigation</t>
+          <t>Transaction</t>
         </is>
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>600</t>
         </is>
       </c>
       <c r="G94" s="5" t="inlineStr">
@@ -4136,12 +4537,17 @@
       </c>
       <c r="H94" s="5" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I94" s="5" t="inlineStr">
         <is>
-          <t>1.512 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J94" s="5" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -4153,27 +4559,27 @@
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>Khách sạn Tam Đảo</t>
+          <t>Hà Nội Trip</t>
         </is>
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>Lưu trú</t>
+          <t>Di chuyển</t>
         </is>
       </c>
       <c r="D95" s="6" t="inlineStr">
         <is>
-          <t>khách sạn 5 sao tam đảo vĩnh phúc</t>
+          <t>thuê xe limousine hà nội tam đảo</t>
         </is>
       </c>
       <c r="E95" s="6" t="inlineStr">
         <is>
-          <t>Commercial Investigation</t>
+          <t>Transaction</t>
         </is>
       </c>
       <c r="F95" s="6" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>250</t>
         </is>
       </c>
       <c r="G95" s="6" t="inlineStr">
@@ -4183,12 +4589,17 @@
       </c>
       <c r="H95" s="6" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I95" s="6" t="inlineStr">
         <is>
-          <t>1.558 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J95" s="6" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -4200,17 +4611,17 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>Khách sạn Tam Đảo</t>
+          <t>Hà Nội Trip</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>Lưu trú</t>
+          <t>Di chuyển</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>khách sạn 4 sao tam đảo</t>
+          <t>tour ghép hà nội tam đảo</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -4220,7 +4631,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G96" s="5" t="inlineStr">
@@ -4230,12 +4641,17 @@
       </c>
       <c r="H96" s="5" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I96" s="5" t="inlineStr">
         <is>
-          <t>572 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J96" s="5" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -4247,27 +4663,27 @@
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>Khách sạn Tam Đảo</t>
+          <t>Thác Bạc Tam Đảo</t>
         </is>
       </c>
       <c r="C97" s="6" t="inlineStr">
         <is>
-          <t>Lưu trú</t>
+          <t>Địa danh tham quan / Văn hóa - Lịch sử</t>
         </is>
       </c>
       <c r="D97" s="6" t="inlineStr">
         <is>
-          <t>khách sạn 3 sao tam đảo</t>
+          <t>du lịch thác bạc tam đảo</t>
         </is>
       </c>
       <c r="E97" s="6" t="inlineStr">
         <is>
-          <t>Commercial Investigation</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="F97" s="6" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G97" s="6" t="inlineStr">
@@ -4277,12 +4693,17 @@
       </c>
       <c r="H97" s="6" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I97" s="6" t="inlineStr">
         <is>
-          <t>1.228 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J97" s="6" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -4294,17 +4715,17 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>Khách sạn Tam Đảo</t>
+          <t>Tour Tam Đảo</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>Lưu trú</t>
+          <t>Di chuyển</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>khách sạn gia lê tam đảo</t>
+          <t>tour du lịch thiền viện trúc lâm tây thiên</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -4314,7 +4735,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>300</t>
         </is>
       </c>
       <c r="G98" s="5" t="inlineStr">
@@ -4324,12 +4745,17 @@
       </c>
       <c r="H98" s="5" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I98" s="5" t="inlineStr">
         <is>
-          <t>1.046 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J98" s="5" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -4341,27 +4767,27 @@
       </c>
       <c r="B99" s="6" t="inlineStr">
         <is>
-          <t>Khách sạn Tam Đảo</t>
+          <t>Tổng hợp Tam Đảo</t>
         </is>
       </c>
       <c r="C99" s="6" t="inlineStr">
         <is>
-          <t>Lưu trú</t>
+          <t>Tổng hợp</t>
         </is>
       </c>
       <c r="D99" s="6" t="inlineStr">
         <is>
-          <t>ngân hà hotel tam đảo</t>
+          <t>hướng dẫn du lịch tam đảo chi tiết</t>
         </is>
       </c>
       <c r="E99" s="6" t="inlineStr">
         <is>
-          <t>Commercial Investigation</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="F99" s="6" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>200</t>
         </is>
       </c>
       <c r="G99" s="6" t="inlineStr">
@@ -4371,12 +4797,17 @@
       </c>
       <c r="H99" s="6" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I99" s="6" t="inlineStr">
         <is>
-          <t>1.933 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J99" s="6" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -4388,17 +4819,17 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>Địa danh Tam Đảo</t>
+          <t>Tổng hợp Tam Đảo</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>Địa danh tham quan</t>
+          <t>Tổng hợp</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>săn mây tam đảo</t>
+          <t>các địa điểm du lịch tam đảo rẻ</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -4408,7 +4839,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>250</t>
         </is>
       </c>
       <c r="G100" s="5" t="inlineStr">
@@ -4418,12 +4849,17 @@
       </c>
       <c r="H100" s="5" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I100" s="5" t="inlineStr">
         <is>
-          <t>317 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J100" s="5" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -4445,7 +4881,7 @@
       </c>
       <c r="D101" s="6" t="inlineStr">
         <is>
-          <t>đi tam đảo mùa nào đẹp nhất</t>
+          <t>địa điểm check in sống ảo tam đảo</t>
         </is>
       </c>
       <c r="E101" s="6" t="inlineStr">
@@ -4465,12 +4901,17 @@
       </c>
       <c r="H101" s="6" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I101" s="6" t="inlineStr">
         <is>
-          <t>253 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J101" s="6" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -4492,7 +4933,7 @@
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>điểm du lịch tam đảo</t>
+          <t>địa điểm ăn ngon tam đảo</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -4502,7 +4943,7 @@
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>400</t>
         </is>
       </c>
       <c r="G102" s="5" t="inlineStr">
@@ -4512,12 +4953,17 @@
       </c>
       <c r="H102" s="5" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I102" s="5" t="inlineStr">
         <is>
-          <t>204 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J102" s="5" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -4529,27 +4975,27 @@
       </c>
       <c r="B103" s="6" t="inlineStr">
         <is>
-          <t>Khách sạn Tam Đảo</t>
+          <t>Tổng hợp Tam Đảo</t>
         </is>
       </c>
       <c r="C103" s="6" t="inlineStr">
         <is>
-          <t>Lưu trú</t>
+          <t>Tổng hợp</t>
         </is>
       </c>
       <c r="D103" s="6" t="inlineStr">
         <is>
-          <t>khách sạn hoàng hà tam đảo</t>
+          <t>du lịch leo núi tam đảo</t>
         </is>
       </c>
       <c r="E103" s="6" t="inlineStr">
         <is>
-          <t>Commercial Investigation</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="F103" s="6" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G103" s="6" t="inlineStr">
@@ -4559,12 +5005,17 @@
       </c>
       <c r="H103" s="6" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I103" s="6" t="inlineStr">
         <is>
-          <t>1.752 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J103" s="6" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -4576,27 +5027,27 @@
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>Khách sạn Tam Đảo</t>
+          <t>Tổng hợp Tam Đảo</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>Lưu trú</t>
+          <t>Tổng hợp</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>khách sạn hương sơn tam đảo</t>
+          <t>địa điểm du lịch mới tam đảo</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t>Commercial Investigation</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="F104" s="5" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>300</t>
         </is>
       </c>
       <c r="G104" s="5" t="inlineStr">
@@ -4606,12 +5057,17 @@
       </c>
       <c r="H104" s="5" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I104" s="5" t="inlineStr">
         <is>
-          <t>1.298 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J104" s="5" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -4623,27 +5079,27 @@
       </c>
       <c r="B105" s="6" t="inlineStr">
         <is>
-          <t>Khách sạn Tam Đảo</t>
+          <t>Tổng hợp Tam Đảo</t>
         </is>
       </c>
       <c r="C105" s="6" t="inlineStr">
         <is>
-          <t>Lưu trú</t>
+          <t>Tổng hợp</t>
         </is>
       </c>
       <c r="D105" s="6" t="inlineStr">
         <is>
-          <t>khách sạn lotus tam đảo</t>
+          <t>du lịch tam đảo 2 ngày 1 đêm tự túc</t>
         </is>
       </c>
       <c r="E105" s="6" t="inlineStr">
         <is>
-          <t>Commercial Investigation</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="F105" s="6" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G105" s="6" t="inlineStr">
@@ -4653,12 +5109,17 @@
       </c>
       <c r="H105" s="6" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I105" s="6" t="inlineStr">
         <is>
-          <t>1.019 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J105" s="6" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -4670,27 +5131,27 @@
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>Đặt phòng Tam Đảo</t>
+          <t>Tổng hợp Tam Đảo</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>Lưu trú</t>
+          <t>Tổng hợp</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>đặt phòng tam đảo giá rẻ</t>
+          <t>kinh nghiệm lịch trình du lịch tam đảo 3 ngày 2 đêm</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t>Transaction</t>
+          <t>Commercial Investigation</t>
         </is>
       </c>
       <c r="F106" s="5" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>300</t>
         </is>
       </c>
       <c r="G106" s="5" t="inlineStr">
@@ -4700,12 +5161,17 @@
       </c>
       <c r="H106" s="5" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I106" s="5" t="inlineStr">
         <is>
-          <t>3.636 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J106" s="5" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -4717,27 +5183,27 @@
       </c>
       <c r="B107" s="6" t="inlineStr">
         <is>
-          <t>Đặt phòng Tam Đảo</t>
+          <t>Tổng hợp Tam Đảo</t>
         </is>
       </c>
       <c r="C107" s="6" t="inlineStr">
         <is>
-          <t>Lưu trú</t>
+          <t>Tổng hợp</t>
         </is>
       </c>
       <c r="D107" s="6" t="inlineStr">
         <is>
-          <t>đặt phòng khách sạn tam đảo</t>
+          <t>kinh nghiệm đặt phòng tam đảo</t>
         </is>
       </c>
       <c r="E107" s="6" t="inlineStr">
         <is>
-          <t>Transaction</t>
+          <t>Commercial Investigation</t>
         </is>
       </c>
       <c r="F107" s="6" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>300</t>
         </is>
       </c>
       <c r="G107" s="6" t="inlineStr">
@@ -4747,12 +5213,17 @@
       </c>
       <c r="H107" s="6" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I107" s="6" t="inlineStr">
         <is>
-          <t>5.436 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J107" s="6" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -4764,27 +5235,27 @@
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>Đặt phòng Tam Đảo</t>
+          <t>Tổng hợp Tam Đảo</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>Lưu trú</t>
+          <t>Tổng hợp</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>đặt khách sạn tại tam đảo</t>
+          <t>kinh nghiệm du lịch bụi tam đảo</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
         <is>
-          <t>Transaction</t>
+          <t>Commercial Investigation</t>
         </is>
       </c>
       <c r="F108" s="5" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>250</t>
         </is>
       </c>
       <c r="G108" s="5" t="inlineStr">
@@ -4794,12 +5265,17 @@
       </c>
       <c r="H108" s="5" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I108" s="5" t="inlineStr">
         <is>
-          <t>12.652 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J108" s="5" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -4811,17 +5287,17 @@
       </c>
       <c r="B109" s="6" t="inlineStr">
         <is>
-          <t>Khách sạn Tam Đảo</t>
+          <t>Vĩnh Phúc Trip</t>
         </is>
       </c>
       <c r="C109" s="6" t="inlineStr">
         <is>
-          <t>Lưu trú</t>
+          <t>Di chuyển</t>
         </is>
       </c>
       <c r="D109" s="6" t="inlineStr">
         <is>
-          <t>khách sạn tam đảo có bể bơi</t>
+          <t>tour du lịch tam đảo vĩnh phúc</t>
         </is>
       </c>
       <c r="E109" s="6" t="inlineStr">
@@ -4831,7 +5307,7 @@
       </c>
       <c r="F109" s="6" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>400</t>
         </is>
       </c>
       <c r="G109" s="6" t="inlineStr">
@@ -4841,12 +5317,17 @@
       </c>
       <c r="H109" s="6" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I109" s="6" t="inlineStr">
         <is>
-          <t>6.079 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J109" s="6" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -4858,27 +5339,27 @@
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>Đặt phòng Tam Đảo</t>
+          <t>Xe buýt đi Tam Đảo</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>Lưu trú</t>
+          <t>Di chuyển</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
         <is>
-          <t>đặt phòng nghỉ ở tam đảo</t>
+          <t>xe bus đi tam đảo rẻ nhất</t>
         </is>
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t>Transaction</t>
+          <t>Commercial Investigation</t>
         </is>
       </c>
       <c r="F110" s="5" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>100</t>
         </is>
       </c>
       <c r="G110" s="5" t="inlineStr">
@@ -4888,12 +5369,17 @@
       </c>
       <c r="H110" s="5" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I110" s="5" t="inlineStr">
         <is>
-          <t>3.964 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J110" s="5" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -4905,27 +5391,27 @@
       </c>
       <c r="B111" s="6" t="inlineStr">
         <is>
-          <t>Tổng hợp Tam Đảo</t>
+          <t>Xe khách đi Tam Đảo</t>
         </is>
       </c>
       <c r="C111" s="6" t="inlineStr">
         <is>
-          <t>Tổng hợp</t>
+          <t>Di chuyển</t>
         </is>
       </c>
       <c r="D111" s="6" t="inlineStr">
         <is>
-          <t>nên ở khách sạn nào ở tam đảo</t>
+          <t>cách di chuyển đi tam đảo bằng xe khách</t>
         </is>
       </c>
       <c r="E111" s="6" t="inlineStr">
         <is>
-          <t>Informational</t>
+          <t>Commercial Investigation</t>
         </is>
       </c>
       <c r="F111" s="6" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G111" s="6" t="inlineStr">
@@ -4935,12 +5421,17 @@
       </c>
       <c r="H111" s="6" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I111" s="6" t="inlineStr">
         <is>
-          <t>1.566 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J111" s="6" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -4952,27 +5443,27 @@
       </c>
       <c r="B112" s="5" t="inlineStr">
         <is>
-          <t>Khách sạn Tam Đảo</t>
+          <t>Xe Limousine đi Tam Đảo</t>
         </is>
       </c>
       <c r="C112" s="5" t="inlineStr">
         <is>
-          <t>Lưu trú</t>
+          <t>Di chuyển</t>
         </is>
       </c>
       <c r="D112" s="5" t="inlineStr">
         <is>
-          <t>đi tam đảo nên ở khách sạn nào</t>
+          <t>xe limousine tam đảo khứ hồi</t>
         </is>
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t>Commercial Investigation</t>
+          <t>Transaction</t>
         </is>
       </c>
       <c r="F112" s="5" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>200</t>
         </is>
       </c>
       <c r="G112" s="5" t="inlineStr">
@@ -4982,12 +5473,17 @@
       </c>
       <c r="H112" s="5" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I112" s="5" t="inlineStr">
         <is>
-          <t>2.078 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J112" s="5" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -4999,27 +5495,27 @@
       </c>
       <c r="B113" s="6" t="inlineStr">
         <is>
-          <t>Đặt phòng Tam Đảo</t>
+          <t>Ăn uống Tam Đảo</t>
         </is>
       </c>
       <c r="C113" s="6" t="inlineStr">
         <is>
-          <t>Lưu trú</t>
+          <t>Ẩm thực (F&amp;B)</t>
         </is>
       </c>
       <c r="D113" s="6" t="inlineStr">
         <is>
-          <t>đặt phòng tại tam đảo</t>
+          <t>nhà hàng buffet nổi tiếng tam đảo</t>
         </is>
       </c>
       <c r="E113" s="6" t="inlineStr">
         <is>
-          <t>Transaction</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="F113" s="6" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>300</t>
         </is>
       </c>
       <c r="G113" s="6" t="inlineStr">
@@ -5029,12 +5525,17 @@
       </c>
       <c r="H113" s="6" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I113" s="6" t="inlineStr">
         <is>
-          <t>4.910 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J113" s="6" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -5046,27 +5547,27 @@
       </c>
       <c r="B114" s="5" t="inlineStr">
         <is>
-          <t>Khách sạn Tam Đảo</t>
+          <t>Ăn uống Tam Đảo</t>
         </is>
       </c>
       <c r="C114" s="5" t="inlineStr">
         <is>
-          <t>Lưu trú</t>
+          <t>Ẩm thực (F&amp;B)</t>
         </is>
       </c>
       <c r="D114" s="5" t="inlineStr">
         <is>
-          <t>top khách sạn tam đảo</t>
+          <t>quán cà phê đẹp tam đảo</t>
         </is>
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t>Commercial Investigation</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="F114" s="5" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>250</t>
         </is>
       </c>
       <c r="G114" s="5" t="inlineStr">
@@ -5076,12 +5577,17 @@
       </c>
       <c r="H114" s="5" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I114" s="5" t="inlineStr">
         <is>
-          <t>3.197 VNĐ</t>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J114" s="5" t="inlineStr">
+        <is>
+          <t>Khác</t>
         </is>
       </c>
     </row>
@@ -5093,27 +5599,27 @@
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
-          <t>Đặt phòng Tam Đảo</t>
+          <t>Ăn uống Tam Đảo</t>
         </is>
       </c>
       <c r="C115" s="6" t="inlineStr">
         <is>
-          <t>Lưu trú</t>
+          <t>Ẩm thực (F&amp;B)</t>
         </is>
       </c>
       <c r="D115" s="6" t="inlineStr">
         <is>
-          <t>đặt phòng ở tam đảo</t>
+          <t>nhà hàng nổi tiếng tam đảo</t>
         </is>
       </c>
       <c r="E115" s="6" t="inlineStr">
         <is>
-          <t>Transaction</t>
+          <t>Informational</t>
         </is>
       </c>
       <c r="F115" s="6" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>150</t>
         </is>
       </c>
       <c r="G115" s="6" t="inlineStr">
@@ -5123,171 +5629,244 @@
       </c>
       <c r="H115" s="6" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>N/A (web)</t>
         </is>
       </c>
       <c r="I115" s="6" t="inlineStr">
         <is>
-          <t>3.292 VNĐ</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="2" t="inlineStr">
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J115" s="6" t="inlineStr">
+        <is>
+          <t>Khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="5" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="B116" s="5" t="inlineStr">
+        <is>
+          <t>Ăn uống Tam Đảo</t>
+        </is>
+      </c>
+      <c r="C116" s="5" t="inlineStr">
+        <is>
+          <t>Ẩm thực (F&amp;B)</t>
+        </is>
+      </c>
+      <c r="D116" s="5" t="inlineStr">
+        <is>
+          <t>quán cà phê check in tam đảo</t>
+        </is>
+      </c>
+      <c r="E116" s="5" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="F116" s="5" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="G116" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H116" s="5" t="inlineStr">
+        <is>
+          <t>N/A (web)</t>
+        </is>
+      </c>
+      <c r="I116" s="5" t="inlineStr">
+        <is>
+          <t>0 VNĐ</t>
+        </is>
+      </c>
+      <c r="J116" s="5" t="inlineStr">
+        <is>
+          <t>Khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
         <is>
           <t>4. CHÚ THÍCH GIẢI NGHĨA CÁC CỘT</t>
         </is>
       </c>
     </row>
-    <row r="119">
-      <c r="A119" s="8" t="inlineStr">
+    <row r="120">
+      <c r="A120" s="8" t="inlineStr">
         <is>
           <t>--- Nhóm A ---</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="9" t="inlineStr">
-        <is>
-          <t>- Cluster: Nhóm chủ đề</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="9" t="inlineStr">
         <is>
-          <t>- Cluster type: Nhóm từ khoá của chủ đề</t>
+          <t>- Cluster: Nhóm chủ đề</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="9" t="inlineStr">
         <is>
-          <t>- Keyword: Từ khoá để SEO</t>
+          <t>- Cluster type: Nhóm từ khoá của chủ đề</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="9" t="inlineStr">
         <is>
-          <t>- Intent: Mục đích, ý định tìm kiếm của khách hàng</t>
+          <t>- Keyword: Từ khoá để SEO</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="9" t="inlineStr">
         <is>
-          <t>- Impression: Số lần Vietgoing hiển thị cho 1 từ khoá cụ thể (Thông thường là ở page 1)</t>
+          <t>- Intent: Mục đích, ý định tìm kiếm của khách hàng</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="9" t="inlineStr">
         <is>
-          <t>- Clicks: Số lượt truy cập vào website Vietgoing cho 1 từ khoá cụ thể</t>
+          <t>- Impression: Số lần Vietgoing hiển thị cho 1 từ khoá cụ thể (Thông thường là ở page 1)</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="9" t="inlineStr">
         <is>
+          <t>- Clicks: Số lượt truy cập vào website Vietgoing cho 1 từ khoá cụ thể</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="9" t="inlineStr">
+        <is>
+          <t>- CTR: Tỷ lệ nhấp chuột (Click-Through Rate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="9" t="inlineStr">
+        <is>
           <t>- Source: Nguồn dữ liệu</t>
         </is>
       </c>
     </row>
-    <row r="128">
-      <c r="A128" s="8" t="inlineStr">
+    <row r="130">
+      <c r="A130" s="8" t="inlineStr">
         <is>
           <t>--- Nhóm B ---</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="9" t="inlineStr">
-        <is>
-          <t>- Cluster: Nhóm chủ đề</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="9" t="inlineStr">
-        <is>
-          <t>- Cluster type: Nhóm từ khoá của chủ đề</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="9" t="inlineStr">
         <is>
-          <t>- Keyword: Từ khoá để SEO</t>
+          <t>- Cluster: Nhóm chủ đề</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="9" t="inlineStr">
         <is>
-          <t>- Intent: Mục đích, ý định tìm kiếm của khách hàng</t>
+          <t>- Cluster type: Nhóm từ khoá của chủ đề</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="9" t="inlineStr">
         <is>
-          <t>- Vol: Lưu lượng tìm kiếm của từ khoá</t>
+          <t>- Keyword: Từ khoá để SEO</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="9" t="inlineStr">
         <is>
-          <t>- YoY: Tăng trưởng tìm kiếm của từ khoá</t>
+          <t>- Intent: Mục đích, ý định tìm kiếm của khách hàng</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="9" t="inlineStr">
         <is>
-          <t>- KD/Comp: Tính cạnh tranh cho từ khoá</t>
+          <t>- Vol: Lưu lượng tìm kiếm của từ khoá</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="9" t="inlineStr">
         <is>
+          <t>- YoY: Tăng trưởng tìm kiếm của từ khoá</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="9" t="inlineStr">
+        <is>
+          <t>- KD/Comp: Tính cạnh tranh cho từ khoá</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="9" t="inlineStr">
+        <is>
           <t>- Bid: Giá thầu dự kiến trên Google Ads (High)</t>
         </is>
       </c>
     </row>
+    <row r="139">
+      <c r="A139" s="9" t="inlineStr">
+        <is>
+          <t>- Source: Nguồn dữ liệu (Google Planner / Seo Insider / Google Trend / Khác)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="28">
-    <mergeCell ref="A7:I7"/>
-    <mergeCell ref="A128:I128"/>
-    <mergeCell ref="A133:I133"/>
-    <mergeCell ref="A118:I118"/>
-    <mergeCell ref="A120:I120"/>
-    <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A136:I136"/>
-    <mergeCell ref="A129:I129"/>
-    <mergeCell ref="A5:I5"/>
-    <mergeCell ref="A126:I126"/>
-    <mergeCell ref="A8:I8"/>
-    <mergeCell ref="A122:I122"/>
-    <mergeCell ref="A135:I135"/>
-    <mergeCell ref="A131:I131"/>
-    <mergeCell ref="A4:I4"/>
-    <mergeCell ref="A62:I62"/>
-    <mergeCell ref="A125:I125"/>
-    <mergeCell ref="A134:I134"/>
-    <mergeCell ref="A121:I121"/>
-    <mergeCell ref="A9:I9"/>
-    <mergeCell ref="A130:I130"/>
-    <mergeCell ref="A11:I11"/>
-    <mergeCell ref="A123:I123"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A132:I132"/>
-    <mergeCell ref="A124:I124"/>
-    <mergeCell ref="A6:I6"/>
-    <mergeCell ref="A119:I119"/>
+  <mergeCells count="30">
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A135:J135"/>
+    <mergeCell ref="A131:J131"/>
+    <mergeCell ref="A126:J126"/>
+    <mergeCell ref="A62:J62"/>
+    <mergeCell ref="A122:J122"/>
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="A125:J125"/>
+    <mergeCell ref="A121:J121"/>
+    <mergeCell ref="A134:J134"/>
+    <mergeCell ref="A127:J127"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="A130:J130"/>
+    <mergeCell ref="A11:J11"/>
+    <mergeCell ref="A138:J138"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A132:J132"/>
+    <mergeCell ref="A123:J123"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A119:J119"/>
+    <mergeCell ref="A124:J124"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A137:J137"/>
+    <mergeCell ref="A128:J128"/>
+    <mergeCell ref="A133:J133"/>
+    <mergeCell ref="A120:J120"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A136:J136"/>
+    <mergeCell ref="A139:J139"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>